<commit_message>
Agenda: colores por estado en toda la fila, varios correos por sede e invitacion al personal, guia de correos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agenda-backend/Agenda_Dr_Rivas_PLANTILLA.xlsx
+++ b/agenda-backend/Agenda_Dr_Rivas_PLANTILLA.xlsx
@@ -125,26 +125,59 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
       <font>
-        <strike val="1"/>
-        <color rgb="009A9A9A"/>
+        <color rgb="005B4B00"/>
       </font>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00E8F3EA"/>
-          <bgColor rgb="00E8F3EA"/>
+          <fgColor rgb="00FFF4CC"/>
+          <bgColor rgb="00FFF4CC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="0012365F"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFF7E0"/>
-          <bgColor rgb="00FFF7E0"/>
+          <fgColor rgb="00DCEBFF"/>
+          <bgColor rgb="00DCEBFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="0014532D"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D3EFD8"/>
+          <bgColor rgb="00D3EFD8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="006B6B6B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E6E6E6"/>
+          <bgColor rgb="00E6E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="008A2F27"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F8D7D3"/>
+          <bgColor rgb="00F8D7D3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -567,7 +600,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>• Cambia la columna "Estado": Pendiente → Confirmada / Atendida / No asistió / Cancelada.</t>
+          <t>• Cambia la columna "Estado": Pendiente (amarillo) → Confirmada (azul) / Atendida (verde) / No asistió (gris) / Cancelada (rojo). La fila completa cambia de color.</t>
         </is>
       </c>
     </row>
@@ -6724,13 +6757,19 @@
   <autoFilter ref="A1:M1000"/>
   <conditionalFormatting sqref="A2:M1000">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$J2="Cancelada"</formula>
+      <formula>$J2="Pendiente"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>$J2="Confirmada"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>$J2="Pendiente"</formula>
+      <formula>$J2="Atendida"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>$J2="No asistió"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="4">
+      <formula>$J2="Cancelada"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -6843,6 +6882,18 @@
       </c>
       <c r="B9" s="10" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Invitar a los correos de la sede al evento de calendario (SI/NO)</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -6863,7 +6914,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Correo que recibe los avisos de la sede</t>
+          <t>Correo(s) de la sede: reciben el aviso de cada cita y la invitación de calendario (separa varios con coma)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">

</xml_diff>